<commit_message>
Add interactive Excel model; fix batch ID leading zeros, ABC tie-break and post-breakdown pallet weight
</commit_message>
<xml_diff>
--- a/outputs/02_storage_requirement.xlsx
+++ b/outputs/02_storage_requirement.xlsx
@@ -1086,8 +1086,10 @@
           <t>PH10031</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>3118120</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>03118120</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1104,8 +1106,10 @@
           <t>PH10031</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>3196802</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>03196802</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1122,8 +1126,10 @@
           <t>PH10044</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>4419147</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>04419147</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1140,8 +1146,10 @@
           <t>PH10044</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>4473643</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>04473643</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1158,8 +1166,10 @@
           <t>PH10044</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>4462709</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04462709</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1176,8 +1186,10 @@
           <t>PH10052</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>5264089</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>05264089</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1194,8 +1206,10 @@
           <t>PH10052</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>5257891</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>05257891</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1212,8 +1226,10 @@
           <t>PH10052</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>5238820</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>05238820</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1230,8 +1246,10 @@
           <t>PH10147</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>14712940</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14712940</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1248,8 +1266,10 @@
           <t>PH10304</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>30430691</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>30430691</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1266,8 +1286,10 @@
           <t>PH10304</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>30411899</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>30411899</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1284,8 +1306,10 @@
           <t>PH10337</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>33750955</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>33750955</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1302,8 +1326,10 @@
           <t>PH10337</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>33753828</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>33753828</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1320,8 +1346,10 @@
           <t>PH10341</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>34199558</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>34199558</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1338,8 +1366,10 @@
           <t>PH10341</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>34123146</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>34123146</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1356,8 +1386,10 @@
           <t>PH10454</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>45430201</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>45430201</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1374,8 +1406,10 @@
           <t>PH10454</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>45470342</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>45470342</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1392,8 +1426,10 @@
           <t>PH10473</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>47378742</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>47378742</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1410,8 +1446,10 @@
           <t>PH10473</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>47399219</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>47399219</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1428,8 +1466,10 @@
           <t>PH10473</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>47352089</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>47352089</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1446,8 +1486,10 @@
           <t>PH10474</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>47445761</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>47445761</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1464,8 +1506,10 @@
           <t>PH10488</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>48819908</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>48819908</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1482,8 +1526,10 @@
           <t>PH10488</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>48895687</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>48895687</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1500,8 +1546,10 @@
           <t>SG20050</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>5091853</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>05091853</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1518,8 +1566,10 @@
           <t>SG20050</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>5061499</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>05061499</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>

</xml_diff>